<commit_message>
Back to questionnaireLabel w&o multilanguage
</commit_message>
<xml_diff>
--- a/tmp/excel/datamodel.xlsx
+++ b/tmp/excel/datamodel.xlsx
@@ -23,13 +23,12 @@
     <sheet name="Answer" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="OrderedQuestion" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Question" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="QuestionRepresentation" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Questionnaire" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="OrderedSection" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Section" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="ScoreDefinition" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="ScoreParameter" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="ScoreValue" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Questionnaire" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="OrderedSection" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Section" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="ScoreDefinition" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="ScoreParameter" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="ScoreValue" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -788,37 +787,37 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>questionHasQuestionRepresentation</t>
+          <t>questionAuthoredByOrg</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>questionAuthoredByOrg</t>
+          <t>questionInOrderedQuestion</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>questionInOrderedQuestion</t>
+          <t>questionHasAnswer</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>questionHasAnswer</t>
+          <t>questionUsedInScoreDefinition</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>questionUsedInScoreDefinition</t>
+          <t>questionId</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>questionId</t>
+          <t>questionTag</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>questionTag</t>
+          <t>questionLabel</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -858,42 +857,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>questionRepresentationOfQuestion</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>questionRepresentationId</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>questionRepresentationText</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>questionRepresentationLanguage</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -959,39 +922,85 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>orderedSectionHasSection</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>orderedSectionPartOfQuestionnaire</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>orderedSectionPartOfSection</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>orderedSectionId</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sectionOrder</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>orderedSectionHasSection</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>orderedSectionPartOfQuestionnaire</t>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sectionHasOrderedQuestion</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sectionHasOrderedSection</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>orderedSectionPartOfSection</t>
+          <t>sectionInOrderedSection</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>orderedSectionId</t>
+          <t>sectionAuthoredByOrg</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>sectionOrder</t>
+          <t>sectionId</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sectionLabel</t>
         </is>
       </c>
     </row>
@@ -1032,52 +1041,6 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>sectionHasOrderedQuestion</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sectionHasOrderedSection</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sectionInOrderedSection</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>sectionAuthoredByOrg</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>sectionId</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>sectionLabel</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1153,7 +1116,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1204,7 +1167,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
scoreDef to Q & S except ex
</commit_message>
<xml_diff>
--- a/tmp/excel/datamodel.xlsx
+++ b/tmp/excel/datamodel.xlsx
@@ -857,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -878,35 +878,40 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>questionnaireUsesScoreDefinition</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>questionnaireAuthoredByOrg</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>questionnairePartOfProcedure</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>questionnaireId</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>questionnaireLabel</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>questionnaireStatus</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>questionnaireVersion</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>questionnaireLastUpdated</t>
         </is>
@@ -914,7 +919,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"draft,active,retired,unknown"</formula1>
     </dataValidation>
   </dataValidations>
@@ -969,7 +974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -990,117 +995,132 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>sectionUsesScoreDefinition</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>sectionAuthoredByOrg</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sectionId</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>sectionLabel</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>first_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>middle_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>family_name</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>scoreDefinitionType</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>scoreDefinitionHasScoreParameter</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>scoreDefinitionUsesQuestion</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>scoreDefinitionHasScoreValue</t>
+        </is>
+      </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>sectionId</t>
+          <t>scoreDefinitionAuthoredByOrg</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>sectionLabel</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>first_name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>middle_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>family_name</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>scoreDefinitionType</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>scoreDefinitionHasScoreParameter</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>scoreDefinitionUsesQuestion</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>scoreDefinitionHasScoreValue</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>scoreDefinitionAuthoredByOrg</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
+          <t>scoreDefinitionUsedByQuestionnare</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>scoreDefinitionUsedBySection</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>scoreDefinitionId</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>scoreDefinitionLabel</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>scoreDefinitionIntervalParams</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>scoreDefinitionFormula</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>scoreDefinitionCategories</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>scoreDefinitionInterpretationGuide</t>
         </is>

</xml_diff>